<commit_message>
Updates analysis XLSX in reference data set.
</commit_message>
<xml_diff>
--- a/data/reference/output/export.202503.categorized.analysis.xlsx
+++ b/data/reference/output/export.202503.categorized.analysis.xlsx
@@ -178,6 +178,64 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Income by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!B13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$A$14:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$14:$B$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Expenses by Category</a:t>
             </a:r>
           </a:p>
@@ -192,7 +250,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!C13</f>
+              <f>'Overview'!B22</f>
             </strRef>
           </tx>
           <spPr>
@@ -202,12 +260,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$14:$A$21</f>
+              <f>'Overview'!$A$23:$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$C$14:$C$21</f>
+              <f>'Overview'!$B$23:$B$30</f>
             </numRef>
           </val>
         </ser>
@@ -227,12 +285,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>3</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="4320000"/>
+    <ext cx="5040000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -242,6 +300,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -539,13 +619,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -576,7 +654,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>8754.299999999999</v>
+        <v>8754.300000000001</v>
       </c>
     </row>
     <row r="7">
@@ -586,7 +664,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2978.09</v>
+        <v>2990.49</v>
       </c>
     </row>
     <row r="8">
@@ -596,13 +674,13 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5776.209999999999</v>
+        <v>5763.810000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Category Breakdown</t>
+          <t>Income by Category</t>
         </is>
       </c>
     </row>
@@ -614,146 +692,127 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Income (CHF)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Expenses (CHF)</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Net (CHF)</t>
+          <t>Amount (CHF)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>8754.299999999999</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>261.29</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>8493.01</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Überträge</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>1787.95</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Expenses by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="4" t="n">
+      <c r="B23" s="4" t="n">
         <v>1825.6</v>
       </c>
-      <c r="D15" s="4" t="n">
-        <v>-1825.6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Überträge</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>23.95</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>433.55</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Einkaufen</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>365.7</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>-365.7</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>233.55</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>-233.55</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="B26" s="4" t="n">
+        <v>382.59</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>130.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Mobilität</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="4" t="n">
+      <c r="B28" s="4" t="n">
         <v>96.90000000000001</v>
       </c>
-      <c r="D18" s="4" t="n">
-        <v>-96.90000000000001</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>-91.09999999999999</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Finanzen</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>-80</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Überträge</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>23.95</v>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>-23.95</v>
+      <c r="B29" s="4" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Uncategorized</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>12.4</v>
       </c>
     </row>
   </sheetData>
@@ -768,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -809,17 +868,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8754.299999999999</v>
+        <v>6966.35</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>261.29</v>
+        <v>0</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>8493.01</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="5">
@@ -841,17 +900,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Überträge</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>365.7</v>
+        <v>23.95</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>-365.7</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="7">
@@ -864,26 +923,26 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>233.55</v>
+        <v>433.55</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>-233.55</v>
+        <v>-433.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>382.59</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-382.59</v>
       </c>
     </row>
     <row r="9">
@@ -896,42 +955,58 @@
         <v>0</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>91.09999999999999</v>
+        <v>130.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-91.09999999999999</v>
+        <v>-130.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>80</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>-80</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>23.95</v>
+        <v>85</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-23.95</v>
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Uncategorized</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>-12.4</v>
       </c>
     </row>
   </sheetData>
@@ -945,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1025,10 +1100,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>150.4</v>
+        <v>167.29</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-150.4</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="6">
@@ -1055,85 +1130,85 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-80</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>91.09999999999999</v>
+        <v>80</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-91.09999999999999</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>101.85</v>
+        <v>5</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-101.85</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>130.5</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-79.90000000000001</v>
+        <v>-130.5</v>
       </c>
     </row>
     <row r="11">
@@ -1144,79 +1219,142 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>51.8</v>
+        <v>200</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-51.8</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>101.85</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-101.85</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nebenkosten</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>1774</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-1774</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sonstiges Leben</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>-51.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Öffentlicher Verkehr</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nebenkosten</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Kommunikation</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4" t="n">
         <v>51.6</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>-51.6</v>
       </c>
     </row>

</xml_diff>